<commit_message>
Point the Week 4 worksheet instructions at the new games
The three Thursday sheets now run datasets the Tuesday lecture never shows, so the
README had to name them. Sheet 1 is Indiana at Los Angeles, where the team that shot
far better lost, and the task is to find the factor that made up the difference.
Sheet 2 is three hitters the deck does not discuss, with on-base and OPS added to the
compute order so the ranking exercise has three rates to disagree about. Sheet 3 is
Baltimore at Buffalo with the score each play was run at, which is what explains the
EPA and WPA disagreement.
</commit_message>
<xml_diff>
--- a/weeks/week04/data/hand-build-descriptive-worksheet.xlsx
+++ b/weeks/week04/data/hand-build-descriptive-worksheet.xlsx
@@ -476,7 +476,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WNBA Finals, Game 3, October 16, 2024. Minnesota Lynx 77, New York Liberty 80, overtime.</t>
+          <t>Fever at Sparks, August 29, 2025. Los Angeles Sparks 75, Indiana Fever 76.</t>
         </is>
       </c>
     </row>
@@ -484,17 +484,17 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>NYL</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Minnesota Lynx</t>
+          <t>Los Angeles Sparks</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -515,10 +515,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C3" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C5" t="n">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -575,10 +575,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -595,10 +595,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -615,10 +615,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C8" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
@@ -635,10 +635,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -648,14 +648,14 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>27</v>
+      </c>
+      <c r="C10" t="n">
         <v>25</v>
       </c>
-      <c r="C10" t="n">
-        <v>27</v>
-      </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>New York Liberty</t>
+          <t>Indiana Fever</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C11" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Every rate on this sheet is built from the counts in B and C, and the two teams share every formula. Fill in MIN, then copy the six formulas down to NYL and check that the references moved with them. The team that made more field goals and turned it over less lost this game; the Four Factors say how.</t>
+          <t>Every rate on this sheet is built from the counts in B and C, and the two teams share every formula. Fill in LAS, then copy the six formulas down to IND and check that the references moved with them. LAS shot better from the field and lost by one. Say which factor made up the difference, and by how much.</t>
         </is>
       </c>
     </row>
@@ -823,15 +823,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -845,25 +846,30 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Arraez</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Judge</t>
+          <t>Rafaela</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Langeliers</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Jonathan India</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -876,18 +882,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>637</v>
+        <v>533</v>
       </c>
       <c r="C3" t="n">
-        <v>559</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+        <v>544</v>
+      </c>
+      <c r="D3" t="n">
+        <v>482</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Singles: hits that were not doubles, triples or home runs</t>
         </is>
       </c>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="5" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -896,18 +905,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>132</v>
       </c>
       <c r="C4" t="n">
-        <v>180</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+        <v>134</v>
+      </c>
+      <c r="D4" t="n">
+        <v>108</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Batting average, H / AB</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="5" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -916,18 +928,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>36</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Slugging, (1B + 2 x 2B + 3 x 3B + 4 x HR) / AB</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="5" t="n"/>
+        <v>23</v>
+      </c>
+      <c r="D5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>On-base %, (H + BB + HBP) / (AB + BB + HBP + SF)</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -936,18 +951,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Unintentional walks, BB - IBB</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="5" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Slugging, (1B + 2 x 2B + 3 x 3B + 4 x HR) / AB</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -956,18 +974,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C7" t="n">
-        <v>58</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>wOBA numerator: each outcome times its weight</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="5" t="n"/>
+        <v>15</v>
+      </c>
+      <c r="D7" t="n">
+        <v>29</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>OPS, on-base plus slugging</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -976,18 +997,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="C8" t="n">
-        <v>133</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>wOBA denominator: AB + uBB + SF + HBP</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="5" t="n"/>
+        <v>15</v>
+      </c>
+      <c r="D8" t="n">
+        <v>41</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Unintentional walks, BB - IBB</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -996,18 +1020,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>20</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>wOBA</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="5" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>wOBA numerator: each outcome times its weight</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1016,11 +1043,21 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>wOBA denominator: AB + uBB + SF + HBP</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1029,35 +1066,38 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Aaron Judge</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>wOBA</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Ceddanne Rafaela</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Singles: hits that were not doubles, triples or home runs</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1065,13 +1105,13 @@
           <t>wOBA weights</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Batting average, H / AB</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="5" t="n"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Singles: hits that were not doubles, triples or home runs</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1082,13 +1122,13 @@
       <c r="B14" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Slugging, (1B + 2 x 2B + 3 x 3B + 4 x HR) / AB</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="5" t="n"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Batting average, H / AB</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1099,13 +1139,13 @@
       <c r="B15" t="n">
         <v>0.72</v>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Unintentional walks, BB - IBB</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="5" t="n"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>On-base %, (H + BB + HBP) / (AB + BB + HBP + SF)</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1116,13 +1156,13 @@
       <c r="B16" t="n">
         <v>0.88</v>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>wOBA numerator: each outcome times its weight</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="5" t="n"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Slugging, (1B + 2 x 2B + 3 x 3B + 4 x HR) / AB</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1133,13 +1173,13 @@
       <c r="B17" t="n">
         <v>1.25</v>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>wOBA denominator: AB + uBB + SF + HBP</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="5" t="n"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>OPS, on-base plus slugging</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1150,13 +1190,13 @@
       <c r="B18" t="n">
         <v>1.58</v>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>wOBA</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="5" t="n"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Unintentional walks, BB - IBB</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1167,83 +1207,271 @@
       <c r="B19" t="n">
         <v>2.01</v>
       </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>wOBA numerator: each outcome times its weight</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Batting average counts every hit once. Slugging weights a hit by the bases it earned. wOBA weights every way of reaching base by the runs it produced, on average, across the league. Fill in Arraez, copy the block down for Judge, and read the three rates side by side.</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>wOBA denominator: AB + uBB + SF + HBP</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>wOBA</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Shea Langeliers</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Your answer</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Singles: hits that were not doubles, triples or home runs</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Batting average, H / AB</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>On-base %, (H + BB + HBP) / (AB + BB + HBP + SF)</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Slugging, (1B + 2 x 2B + 3 x 3B + 4 x HR) / AB</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>OPS, on-base plus slugging</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Unintentional walks, BB - IBB</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>wOBA numerator: each outcome times its weight</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>wOBA denominator: AB + uBB + SF + HBP</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>wOBA</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>Batting average counts every hit once. Slugging weights a hit by the bases it earned. OPS adds on-base percentage to slugging and stops there. wOBA weights every way of reaching base by the runs it produced, on average, across the league. Fill in India, copy the block down for the other two, then rank the three hitters by average, by OPS and by wOBA. Where the rankings disagree, say which one you would trust and whether wOBA's extra work bought anything.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F3">
+  <conditionalFormatting sqref="G3">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(ISNUMBER(E3),ABS(E3-(($B$4-$B$5-$B$6-$B$7)))&lt;=MAX(0.02*ABS(($B$4-$B$5-$B$6-$B$7)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F4">
+      <formula>AND(ISNUMBER(F3),ABS(F3-(($B$4-$B$5-$B$6-$B$7)))&lt;=MAX(0.02*ABS(($B$4-$B$5-$B$6-$B$7)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>AND(ISNUMBER(E4),ABS(E4-(($B$4/$B$3)))&lt;=MAX(0.02*ABS(($B$4/$B$3)),0.002))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F5">
+      <formula>AND(ISNUMBER(F4),ABS(F4-(($B$4/$B$3)))&lt;=MAX(0.02*ABS(($B$4/$B$3)),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>AND(ISNUMBER(E5),ABS(E5-(((($B$4-$B$5-$B$6-$B$7)+2*$B$5+3*$B$6+4*$B$7)/$B$3)))&lt;=MAX(0.02*ABS(((($B$4-$B$5-$B$6-$B$7)+2*$B$5+3*$B$6+4*$B$7)/$B$3)),0.003))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F6">
+      <formula>AND(ISNUMBER(F5),ABS(F5-((($B$4+$B$8+$B$10)/($B$3+$B$8+$B$10+$B$11))))&lt;=MAX(0.02*ABS((($B$4+$B$8+$B$10)/($B$3+$B$8+$B$10+$B$11))),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6">
     <cfRule type="expression" priority="4" dxfId="0">
-      <formula>AND(ISNUMBER(E6),ABS(E6-(($B$8-$B$9)))&lt;=MAX(0.02*ABS(($B$8-$B$9)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7">
+      <formula>AND(ISNUMBER(F6),ABS(F6-(((($B$4-$B$5-$B$6-$B$7)+2*$B$5+3*$B$6+4*$B$7)/$B$3)))&lt;=MAX(0.02*ABS(((($B$4-$B$5-$B$6-$B$7)+2*$B$5+3*$B$6+4*$B$7)/$B$3)),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
     <cfRule type="expression" priority="5" dxfId="0">
-      <formula>AND(ISNUMBER(E7),ABS(E7-(($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)))&lt;=MAX(0.02*ABS(($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F8">
+      <formula>AND(ISNUMBER(F7),ABS(F7-(((($B$4+$B$8+$B$10)/($B$3+$B$8+$B$10+$B$11))+((($B$4-$B$5-$B$6-$B$7)+2*$B$5+3*$B$6+4*$B$7)/$B$3))))&lt;=MAX(0.02*ABS(((($B$4+$B$8+$B$10)/($B$3+$B$8+$B$10+$B$11))+((($B$4-$B$5-$B$6-$B$7)+2*$B$5+3*$B$6+4*$B$7)/$B$3))),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8">
     <cfRule type="expression" priority="6" dxfId="0">
-      <formula>AND(ISNUMBER(E8),ABS(E8-(($B$3+($B$8-$B$9)+$B$11+$B$10)))&lt;=MAX(0.02*ABS(($B$3+($B$8-$B$9)+$B$11+$B$10)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F9">
+      <formula>AND(ISNUMBER(F8),ABS(F8-(($B$8-$B$9)))&lt;=MAX(0.02*ABS(($B$8-$B$9)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
     <cfRule type="expression" priority="7" dxfId="0">
-      <formula>AND(ISNUMBER(E9),ABS(E9-((($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)/($B$3+($B$8-$B$9)+$B$11+$B$10))))&lt;=MAX(0.02*ABS((($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)/($B$3+($B$8-$B$9)+$B$11+$B$10))),0.003))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F12">
+      <formula>AND(ISNUMBER(F9),ABS(F9-(($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)))&lt;=MAX(0.02*ABS(($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10">
     <cfRule type="expression" priority="8" dxfId="0">
-      <formula>AND(ISNUMBER(E12),ABS(E12-(($C$4-$C$5-$C$6-$C$7)))&lt;=MAX(0.02*ABS(($C$4-$C$5-$C$6-$C$7)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F13">
+      <formula>AND(ISNUMBER(F10),ABS(F10-(($B$3+($B$8-$B$9)+$B$11+$B$10)))&lt;=MAX(0.02*ABS(($B$3+($B$8-$B$9)+$B$11+$B$10)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11">
     <cfRule type="expression" priority="9" dxfId="0">
-      <formula>AND(ISNUMBER(E13),ABS(E13-(($C$4/$C$3)))&lt;=MAX(0.02*ABS(($C$4/$C$3)),0.002))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F14">
+      <formula>AND(ISNUMBER(F11),ABS(F11-((($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)/($B$3+($B$8-$B$9)+$B$11+$B$10))))&lt;=MAX(0.02*ABS((($B$14*($B$8-$B$9)+$B$15*$B$10+$B$16*($B$4-$B$5-$B$6-$B$7)+$B$17*$B$5+$B$18*$B$6+$B$19*$B$7)/($B$3+($B$8-$B$9)+$B$11+$B$10))),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G13">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>AND(ISNUMBER(E14),ABS(E14-(((($C$4-$C$5-$C$6-$C$7)+2*$C$5+3*$C$6+4*$C$7)/$C$3)))&lt;=MAX(0.02*ABS(((($C$4-$C$5-$C$6-$C$7)+2*$C$5+3*$C$6+4*$C$7)/$C$3)),0.003))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F15">
+      <formula>AND(ISNUMBER(F13),ABS(F13-(($C$4-$C$5-$C$6-$C$7)))&lt;=MAX(0.02*ABS(($C$4-$C$5-$C$6-$C$7)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G14">
     <cfRule type="expression" priority="11" dxfId="0">
-      <formula>AND(ISNUMBER(E15),ABS(E15-(($C$8-$C$9)))&lt;=MAX(0.02*ABS(($C$8-$C$9)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F16">
+      <formula>AND(ISNUMBER(F14),ABS(F14-(($C$4/$C$3)))&lt;=MAX(0.02*ABS(($C$4/$C$3)),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15">
     <cfRule type="expression" priority="12" dxfId="0">
-      <formula>AND(ISNUMBER(E16),ABS(E16-(($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)))&lt;=MAX(0.02*ABS(($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F17">
+      <formula>AND(ISNUMBER(F15),ABS(F15-((($C$4+$C$8+$C$10)/($C$3+$C$8+$C$10+$C$11))))&lt;=MAX(0.02*ABS((($C$4+$C$8+$C$10)/($C$3+$C$8+$C$10+$C$11))),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(E17),ABS(E17-(($C$3+($C$8-$C$9)+$C$11+$C$10)))&lt;=MAX(0.02*ABS(($C$3+($C$8-$C$9)+$C$11+$C$10)),0.5))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F18">
+      <formula>AND(ISNUMBER(F16),ABS(F16-(((($C$4-$C$5-$C$6-$C$7)+2*$C$5+3*$C$6+4*$C$7)/$C$3)))&lt;=MAX(0.02*ABS(((($C$4-$C$5-$C$6-$C$7)+2*$C$5+3*$C$6+4*$C$7)/$C$3)),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17">
     <cfRule type="expression" priority="14" dxfId="0">
-      <formula>AND(ISNUMBER(E18),ABS(E18-((($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)/($C$3+($C$8-$C$9)+$C$11+$C$10))))&lt;=MAX(0.02*ABS((($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)/($C$3+($C$8-$C$9)+$C$11+$C$10))),0.003))</formula>
+      <formula>AND(ISNUMBER(F17),ABS(F17-(((($C$4+$C$8+$C$10)/($C$3+$C$8+$C$10+$C$11))+((($C$4-$C$5-$C$6-$C$7)+2*$C$5+3*$C$6+4*$C$7)/$C$3))))&lt;=MAX(0.02*ABS(((($C$4+$C$8+$C$10)/($C$3+$C$8+$C$10+$C$11))+((($C$4-$C$5-$C$6-$C$7)+2*$C$5+3*$C$6+4*$C$7)/$C$3))),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18">
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>AND(ISNUMBER(F18),ABS(F18-(($C$8-$C$9)))&lt;=MAX(0.02*ABS(($C$8-$C$9)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19">
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>AND(ISNUMBER(F19),ABS(F19-(($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)))&lt;=MAX(0.02*ABS(($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>AND(ISNUMBER(F20),ABS(F20-(($C$3+($C$8-$C$9)+$C$11+$C$10)))&lt;=MAX(0.02*ABS(($C$3+($C$8-$C$9)+$C$11+$C$10)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G21">
+    <cfRule type="expression" priority="18" dxfId="0">
+      <formula>AND(ISNUMBER(F21),ABS(F21-((($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)/($C$3+($C$8-$C$9)+$C$11+$C$10))))&lt;=MAX(0.02*ABS((($B$14*($C$8-$C$9)+$B$15*$C$10+$B$16*($C$4-$C$5-$C$6-$C$7)+$B$17*$C$5+$B$18*$C$6+$B$19*$C$7)/($C$3+($C$8-$C$9)+$C$11+$C$10))),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23">
+    <cfRule type="expression" priority="19" dxfId="0">
+      <formula>AND(ISNUMBER(F23),ABS(F23-(($D$4-$D$5-$D$6-$D$7)))&lt;=MAX(0.02*ABS(($D$4-$D$5-$D$6-$D$7)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G24">
+    <cfRule type="expression" priority="20" dxfId="0">
+      <formula>AND(ISNUMBER(F24),ABS(F24-(($D$4/$D$3)))&lt;=MAX(0.02*ABS(($D$4/$D$3)),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G25">
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>AND(ISNUMBER(F25),ABS(F25-((($D$4+$D$8+$D$10)/($D$3+$D$8+$D$10+$D$11))))&lt;=MAX(0.02*ABS((($D$4+$D$8+$D$10)/($D$3+$D$8+$D$10+$D$11))),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G26">
+    <cfRule type="expression" priority="22" dxfId="0">
+      <formula>AND(ISNUMBER(F26),ABS(F26-(((($D$4-$D$5-$D$6-$D$7)+2*$D$5+3*$D$6+4*$D$7)/$D$3)))&lt;=MAX(0.02*ABS(((($D$4-$D$5-$D$6-$D$7)+2*$D$5+3*$D$6+4*$D$7)/$D$3)),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G27">
+    <cfRule type="expression" priority="23" dxfId="0">
+      <formula>AND(ISNUMBER(F27),ABS(F27-(((($D$4+$D$8+$D$10)/($D$3+$D$8+$D$10+$D$11))+((($D$4-$D$5-$D$6-$D$7)+2*$D$5+3*$D$6+4*$D$7)/$D$3))))&lt;=MAX(0.02*ABS(((($D$4+$D$8+$D$10)/($D$3+$D$8+$D$10+$D$11))+((($D$4-$D$5-$D$6-$D$7)+2*$D$5+3*$D$6+4*$D$7)/$D$3))),0.003))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28">
+    <cfRule type="expression" priority="24" dxfId="0">
+      <formula>AND(ISNUMBER(F28),ABS(F28-(($D$8-$D$9)))&lt;=MAX(0.02*ABS(($D$8-$D$9)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
+    <cfRule type="expression" priority="25" dxfId="0">
+      <formula>AND(ISNUMBER(F29),ABS(F29-(($B$14*($D$8-$D$9)+$B$15*$D$10+$B$16*($D$4-$D$5-$D$6-$D$7)+$B$17*$D$5+$B$18*$D$6+$B$19*$D$7)))&lt;=MAX(0.02*ABS(($B$14*($D$8-$D$9)+$B$15*$D$10+$B$16*($D$4-$D$5-$D$6-$D$7)+$B$17*$D$5+$B$18*$D$6+$B$19*$D$7)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30">
+    <cfRule type="expression" priority="26" dxfId="0">
+      <formula>AND(ISNUMBER(F30),ABS(F30-(($D$3+($D$8-$D$9)+$D$11+$D$10)))&lt;=MAX(0.02*ABS(($D$3+($D$8-$D$9)+$D$11+$D$10)),0.5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G31">
+    <cfRule type="expression" priority="27" dxfId="0">
+      <formula>AND(ISNUMBER(F31),ABS(F31-((($B$14*($D$8-$D$9)+$B$15*$D$10+$B$16*($D$4-$D$5-$D$6-$D$7)+$B$17*$D$5+$B$18*$D$6+$B$19*$D$7)/($D$3+($D$8-$D$9)+$D$11+$D$10))))&lt;=MAX(0.02*ABS((($B$14*($D$8-$D$9)+$B$15*$D$10+$B$16*($D$4-$D$5-$D$6-$D$7)+$B$17*$D$5+$B$18*$D$6+$B$19*$D$7)/($D$3+($D$8-$D$9)+$D$11+$D$10))),0.003))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1256,26 +1484,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Super Bowl LI, ATL 28, NE 34. 12 of the game's 169 plays. nflverse.</t>
+          <t>Ravens at Bills, Week 1, BUF 41, BAL 40. 12 of the game's 163 plays. nflverse.</t>
         </is>
       </c>
     </row>
@@ -1292,45 +1521,50 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>Play</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>EPA</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>WPA</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>z EPA</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>z WPA</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>z WPA - z EPA</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
@@ -1339,577 +1573,637 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q2 15:00</t>
+          <t>Q2 01:46</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>12-T.Brady pass deep right to 11-J.Edelman to ATL 33 for 27 yards.</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="n">
-        <v>2.314</v>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>0.1014</v>
-      </c>
-      <c r="F3" s="6" t="n"/>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>17-10</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>43-J.Hill left tackle to BUF 23 for -6 yards. FUMBLES, and recovers at BUF 29. 43-J.Hill to BUF 32...</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="n">
+        <v>-2.216</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>-0.0177</v>
+      </c>
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
-      <c r="I3" s="5" t="n"/>
+      <c r="I3" s="6" t="n"/>
       <c r="J3" s="5" t="n"/>
       <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q2 14:19</t>
+          <t>Q3 13:42</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>29-L.Blount left tackle to ATL 29 for 4 yards. FUMBLES, RECOVERED by ATL-23-R.Alford at ATL 29. 23-...</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>-4.922</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>-0.1421</v>
-      </c>
-      <c r="F4" s="6" t="n"/>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>20-13</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>8-L.Jackson pass deep middle to 4-Z.Flowers to BUF 23 for 39 yards.</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>4.151</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>0.097</v>
+      </c>
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="n"/>
-      <c r="I4" s="5" t="n"/>
+      <c r="I4" s="6" t="n"/>
       <c r="J4" s="5" t="n"/>
       <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q2 02:36</t>
+          <t>Q3 01:14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>12-T.Brady pass short left intended for 80-D.Amendola INTERCEPTED by 23-R.Alford at ATL 18. 23-R.Al...</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>-10.186</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>-0.0975</v>
-      </c>
-      <c r="F5" s="6" t="n"/>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>27-19</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>8-L.Jackson pass deep right to 10-D.Hopkins for 29 yards, TOUCHDOWN.</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>3.422</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>0.0529</v>
+      </c>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
-      <c r="I5" s="5" t="n"/>
+      <c r="I5" s="6" t="n"/>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q3 11:36</t>
+          <t>Q4 14:06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ATL</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>2-M.Ryan pass deep middle to 18-T.Gabriel to NE 28 for 35 yards.</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>2.807</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>0.0061</v>
-      </c>
-      <c r="F6" s="6" t="n"/>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>19-34</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>17-J.Allen pass short right to 4-J.Cook to BAL 2 for 51 yards.</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>4.995</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0.0641</v>
+      </c>
       <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
-      <c r="I6" s="5" t="n"/>
+      <c r="I6" s="6" t="n"/>
       <c r="J6" s="5" t="n"/>
       <c r="K6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Q3 06:04</t>
+          <t>Q4 11:50</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>12-T.Brady pass short left to 80-D.Amendola pushed ob at ATL 37 for 17 yards.</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>4.059</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F7" s="6" t="n"/>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>34-25</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>22-D.Henry left tackle for 46 yards, TOUCHDOWN.</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0.0466</v>
+      </c>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
-      <c r="I7" s="5" t="n"/>
+      <c r="I7" s="6" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Q4 08:31</t>
+          <t>Q4 04:05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ATL</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>2-M.Ryan sacked at ATL 25 for -11 yards. FUMBLES, RECOVERED by NE-97-A.Branch at ATL 25. 97-A.Branc...</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>-5.7</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>-0.0386</v>
-      </c>
-      <c r="F8" s="6" t="n"/>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>25-40</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>17-J.Allen pass short right to 0-K.Coleman for 10 yards, TOUCHDOWN.</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>3.997</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0.0184</v>
+      </c>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="I8" s="6" t="n"/>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Q4 01:00</t>
+          <t>Q4 03:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>28-J.White right guard for 1 yard, TOUCHDOWN.</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>1.779</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>-0.0244</v>
-      </c>
-      <c r="F9" s="6" t="n"/>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>40-32</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>66-B.Cleveland reported in as eligible. 22-D.Henry left tackle to BAL 38 for -3 yards. FUMBLES, tou...</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>-5.282</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>-0.0893</v>
+      </c>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
-      <c r="I9" s="5" t="n"/>
+      <c r="I9" s="6" t="n"/>
       <c r="J9" s="5" t="n"/>
       <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Q4 00:18</t>
+          <t>Q4 01:58</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ATL</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>2-M.Ryan pass incomplete deep left to 81-A.Hooper.</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>-0.079</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>-0.0941</v>
-      </c>
-      <c r="F10" s="6" t="n"/>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>38-40</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>TWO-POINT CONVERSION ATTEMPT. 17-J.Allen pass to 0-K.Coleman is incomplete. ATTEMPT FAILS.</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>-0.947</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>-0.1411</v>
+      </c>
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="6" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="I10" s="6" t="n"/>
       <c r="J10" s="5" t="n"/>
       <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>OT 14:26</t>
+          <t>Q4 01:33</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>12-T.Brady pass short right to 80-D.Amendola ran ob at NE 45 for 14 yards.</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="n">
-        <v>1.057</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>0.1082</v>
-      </c>
-      <c r="F11" s="6" t="n"/>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>40-38</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>11-J.Stout punts 42 yards to BUF 20, Center-46-N.Moore, out of bounds.</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>-0.304</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>-0.2096</v>
+      </c>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="I11" s="6" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>OT 13:59</t>
+          <t>Q4 00:53</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>12-T.Brady pass short left to 15-C.Hogan to ATL 37 for 18 yards.</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="n">
-        <v>1.241</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>0.1388</v>
-      </c>
-      <c r="F12" s="6" t="n"/>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>38-40</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>17-J.Allen pass deep left to 5-J.Palmer ran ob at BAL 34 for 32 yards.</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>2.219</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.1896</v>
+      </c>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
-      <c r="I12" s="5" t="n"/>
+      <c r="I12" s="6" t="n"/>
       <c r="J12" s="5" t="n"/>
       <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OT 13:12</t>
+          <t>Q4 00:46</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>12-T.Brady pass short left to 28-J.White to ATL 40 for -3 yards.</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>-1.088</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>-0.0956</v>
-      </c>
-      <c r="F13" s="6" t="n"/>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>38-40</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>17-J.Allen pass short middle to 0-K.Coleman to BAL 9 for 25 yards.</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>1.897</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0.197</v>
+      </c>
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="6" t="n"/>
-      <c r="I13" s="5" t="n"/>
+      <c r="I13" s="6" t="n"/>
       <c r="J13" s="5" t="n"/>
       <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>OT 12:37</t>
+          <t>Q4 00:03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>12-T.Brady pass short left to 11-J.Edelman to ATL 25 for 15 yards.</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>1.801</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>0.1646</v>
-      </c>
-      <c r="F14" s="6" t="n"/>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>38-40</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>15-M.Prater 32 yard field goal is GOOD, Center-69-R.Ferguson, Holder-40-B.Robbins.</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0.3854</v>
+      </c>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
-      <c r="I14" s="5" t="n"/>
+      <c r="I14" s="6" t="n"/>
       <c r="J14" s="5" t="n"/>
       <c r="K14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Correlation between EPA and WPA across these plays, CORREL</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="5" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="C18" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Largest disagreement, ignoring sign: MAX of the absolute values</t>
         </is>
       </c>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="5" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>STANDARDIZE(x, mean, standard deviation) puts EPA and WPA on the same scale so they can be compared. A positive number in the last column is a play that mattered more to the win than to the score; a negative one is the reverse. Find the two biggest, in either direction, and say what they have in common.</t>
+          <t>STANDARDIZE(x, mean, standard deviation) puts EPA and WPA on the same scale so they can be compared. A positive number in the last column is a play that mattered more to the win than to the score; a negative one is the reverse. Find the two biggest, in either direction, look at the score column next to them, and say what they have in common.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I3">
+  <conditionalFormatting sqref="J3">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(ISNUMBER(F3),ABS(F3-(STANDARDIZE($D3,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D3,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J3">
+      <formula>AND(ISNUMBER(G3),ABS(G3-(STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>AND(ISNUMBER(G3),ABS(G3-(STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3">
+      <formula>AND(ISNUMBER(H3),ABS(H3-(STANDARDIZE($F3,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F3,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>AND(ISNUMBER(H3),ABS(H3-((STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D3,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D3,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4">
+      <formula>AND(ISNUMBER(I3),ABS(I3-((STANDARDIZE($F3,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F3,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E3,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4">
     <cfRule type="expression" priority="4" dxfId="0">
-      <formula>AND(ISNUMBER(F4),ABS(F4-(STANDARDIZE($D4,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D4,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J4">
+      <formula>AND(ISNUMBER(G4),ABS(G4-(STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4">
     <cfRule type="expression" priority="5" dxfId="0">
-      <formula>AND(ISNUMBER(G4),ABS(G4-(STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K4">
+      <formula>AND(ISNUMBER(H4),ABS(H4-(STANDARDIZE($F4,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F4,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L4">
     <cfRule type="expression" priority="6" dxfId="0">
-      <formula>AND(ISNUMBER(H4),ABS(H4-((STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D4,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D4,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I5">
+      <formula>AND(ISNUMBER(I4),ABS(I4-((STANDARDIZE($F4,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F4,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E4,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5">
     <cfRule type="expression" priority="7" dxfId="0">
-      <formula>AND(ISNUMBER(F5),ABS(F5-(STANDARDIZE($D5,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D5,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5">
+      <formula>AND(ISNUMBER(G5),ABS(G5-(STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5">
     <cfRule type="expression" priority="8" dxfId="0">
-      <formula>AND(ISNUMBER(G5),ABS(G5-(STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K5">
+      <formula>AND(ISNUMBER(H5),ABS(H5-(STANDARDIZE($F5,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F5,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5">
     <cfRule type="expression" priority="9" dxfId="0">
-      <formula>AND(ISNUMBER(H5),ABS(H5-((STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D5,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D5,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I6">
+      <formula>AND(ISNUMBER(I5),ABS(I5-((STANDARDIZE($F5,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F5,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E5,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>AND(ISNUMBER(F6),ABS(F6-(STANDARDIZE($D6,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D6,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J6">
+      <formula>AND(ISNUMBER(G6),ABS(G6-(STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6">
     <cfRule type="expression" priority="11" dxfId="0">
-      <formula>AND(ISNUMBER(G6),ABS(G6-(STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K6">
+      <formula>AND(ISNUMBER(H6),ABS(H6-(STANDARDIZE($F6,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F6,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L6">
     <cfRule type="expression" priority="12" dxfId="0">
-      <formula>AND(ISNUMBER(H6),ABS(H6-((STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D6,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D6,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7">
+      <formula>AND(ISNUMBER(I6),ABS(I6-((STANDARDIZE($F6,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F6,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E6,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(F7),ABS(F7-(STANDARDIZE($D7,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D7,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7">
+      <formula>AND(ISNUMBER(G7),ABS(G7-(STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7">
     <cfRule type="expression" priority="14" dxfId="0">
-      <formula>AND(ISNUMBER(G7),ABS(G7-(STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7">
+      <formula>AND(ISNUMBER(H7),ABS(H7-(STANDARDIZE($F7,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F7,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7">
     <cfRule type="expression" priority="15" dxfId="0">
-      <formula>AND(ISNUMBER(H7),ABS(H7-((STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D7,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D7,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8">
+      <formula>AND(ISNUMBER(I7),ABS(I7-((STANDARDIZE($F7,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F7,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E7,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J8">
     <cfRule type="expression" priority="16" dxfId="0">
-      <formula>AND(ISNUMBER(F8),ABS(F8-(STANDARDIZE($D8,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D8,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J8">
+      <formula>AND(ISNUMBER(G8),ABS(G8-(STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K8">
     <cfRule type="expression" priority="17" dxfId="0">
-      <formula>AND(ISNUMBER(G8),ABS(G8-(STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K8">
+      <formula>AND(ISNUMBER(H8),ABS(H8-(STANDARDIZE($F8,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F8,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L8">
     <cfRule type="expression" priority="18" dxfId="0">
-      <formula>AND(ISNUMBER(H8),ABS(H8-((STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D8,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D8,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I9">
+      <formula>AND(ISNUMBER(I8),ABS(I8-((STANDARDIZE($F8,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F8,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E8,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J9">
     <cfRule type="expression" priority="19" dxfId="0">
-      <formula>AND(ISNUMBER(F9),ABS(F9-(STANDARDIZE($D9,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D9,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J9">
+      <formula>AND(ISNUMBER(G9),ABS(G9-(STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9">
     <cfRule type="expression" priority="20" dxfId="0">
-      <formula>AND(ISNUMBER(G9),ABS(G9-(STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K9">
+      <formula>AND(ISNUMBER(H9),ABS(H9-(STANDARDIZE($F9,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F9,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L9">
     <cfRule type="expression" priority="21" dxfId="0">
-      <formula>AND(ISNUMBER(H9),ABS(H9-((STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D9,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D9,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10">
+      <formula>AND(ISNUMBER(I9),ABS(I9-((STANDARDIZE($F9,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F9,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E9,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J10">
     <cfRule type="expression" priority="22" dxfId="0">
-      <formula>AND(ISNUMBER(F10),ABS(F10-(STANDARDIZE($D10,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D10,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J10">
+      <formula>AND(ISNUMBER(G10),ABS(G10-(STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K10">
     <cfRule type="expression" priority="23" dxfId="0">
-      <formula>AND(ISNUMBER(G10),ABS(G10-(STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K10">
+      <formula>AND(ISNUMBER(H10),ABS(H10-(STANDARDIZE($F10,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F10,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L10">
     <cfRule type="expression" priority="24" dxfId="0">
-      <formula>AND(ISNUMBER(H10),ABS(H10-((STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D10,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D10,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I11">
+      <formula>AND(ISNUMBER(I10),ABS(I10-((STANDARDIZE($F10,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F10,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E10,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11">
     <cfRule type="expression" priority="25" dxfId="0">
-      <formula>AND(ISNUMBER(F11),ABS(F11-(STANDARDIZE($D11,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D11,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11">
+      <formula>AND(ISNUMBER(G11),ABS(G11-(STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
     <cfRule type="expression" priority="26" dxfId="0">
-      <formula>AND(ISNUMBER(G11),ABS(G11-(STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K11">
+      <formula>AND(ISNUMBER(H11),ABS(H11-(STANDARDIZE($F11,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F11,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L11">
     <cfRule type="expression" priority="27" dxfId="0">
-      <formula>AND(ISNUMBER(H11),ABS(H11-((STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D11,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D11,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I12">
+      <formula>AND(ISNUMBER(I11),ABS(I11-((STANDARDIZE($F11,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F11,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E11,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J12">
     <cfRule type="expression" priority="28" dxfId="0">
-      <formula>AND(ISNUMBER(F12),ABS(F12-(STANDARDIZE($D12,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D12,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J12">
+      <formula>AND(ISNUMBER(G12),ABS(G12-(STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12">
     <cfRule type="expression" priority="29" dxfId="0">
-      <formula>AND(ISNUMBER(G12),ABS(G12-(STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K12">
+      <formula>AND(ISNUMBER(H12),ABS(H12-(STANDARDIZE($F12,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F12,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L12">
     <cfRule type="expression" priority="30" dxfId="0">
-      <formula>AND(ISNUMBER(H12),ABS(H12-((STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D12,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D12,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I13">
+      <formula>AND(ISNUMBER(I12),ABS(I12-((STANDARDIZE($F12,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F12,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E12,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J13">
     <cfRule type="expression" priority="31" dxfId="0">
-      <formula>AND(ISNUMBER(F13),ABS(F13-(STANDARDIZE($D13,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D13,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J13">
+      <formula>AND(ISNUMBER(G13),ABS(G13-(STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K13">
     <cfRule type="expression" priority="32" dxfId="0">
-      <formula>AND(ISNUMBER(G13),ABS(G13-(STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K13">
+      <formula>AND(ISNUMBER(H13),ABS(H13-(STANDARDIZE($F13,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F13,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L13">
     <cfRule type="expression" priority="33" dxfId="0">
-      <formula>AND(ISNUMBER(H13),ABS(H13-((STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D13,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D13,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I14">
+      <formula>AND(ISNUMBER(I13),ABS(I13-((STANDARDIZE($F13,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F13,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E13,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J14">
     <cfRule type="expression" priority="34" dxfId="0">
-      <formula>AND(ISNUMBER(F14),ABS(F14-(STANDARDIZE($D14,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($D14,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J14">
+      <formula>AND(ISNUMBER(G14),ABS(G14-(STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K14">
     <cfRule type="expression" priority="35" dxfId="0">
-      <formula>AND(ISNUMBER(G14),ABS(G14-(STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K14">
+      <formula>AND(ISNUMBER(H14),ABS(H14-(STANDARDIZE($F14,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))))&lt;=MAX(0.02*ABS(STANDARDIZE($F14,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L14">
     <cfRule type="expression" priority="36" dxfId="0">
-      <formula>AND(ISNUMBER(H14),ABS(H14-((STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D14,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14))-STANDARDIZE($D14,AVERAGE($D$3:$D$14),_xlfn.STDEV.S($D$3:$D$14)))),0.02))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17">
+      <formula>AND(ISNUMBER(I14),ABS(I14-((STANDARDIZE($F14,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))))&lt;=MAX(0.02*ABS((STANDARDIZE($F14,AVERAGE($F$3:$F$14),_xlfn.STDEV.S($F$3:$F$14))-STANDARDIZE($E14,AVERAGE($E$3:$E$14),_xlfn.STDEV.S($E$3:$E$14)))),0.02))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17">
     <cfRule type="expression" priority="37" dxfId="0">
-      <formula>AND(ISNUMBER(D17),ABS(D17-(CORREL(D3:D14,E3:E14)))&lt;=MAX(0.02*ABS(CORREL(D3:D14,E3:E14)),0.01))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
+      <formula>AND(ISNUMBER(E17),ABS(E17-(CORREL(E3:E14,F3:F14)))&lt;=MAX(0.02*ABS(CORREL(E3:E14,F3:F14)),0.01))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F18">
     <cfRule type="expression" priority="38" dxfId="0">
-      <formula>AND(ISNUMBER(D18),ABS(D18-(MAX(ABS(MIN(H3:H14)),MAX(H3:H14))))&lt;=MAX(0.02*ABS(MAX(ABS(MIN(H3:H14)),MAX(H3:H14))),0.02))</formula>
+      <formula>AND(ISNUMBER(E18),ABS(E18-(MAX(ABS(MIN(I3:I14)),MAX(I3:I14))))&lt;=MAX(0.02*ABS(MAX(ABS(MIN(I3:I14)),MAX(I3:I14))),0.02))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Show one percent sign on the four-factors labels
The eFG, turnover and offensive rebound rows read with a doubled percent sign,
which looked like a typo in the sheet students are asked to trust.
</commit_message>
<xml_diff>
--- a/weeks/week04/data/hand-build-descriptive-worksheet.xlsx
+++ b/weeks/week04/data/hand-build-descriptive-worksheet.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>eFG%%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
+          <t>eFG%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
         </is>
       </c>
       <c r="E3" s="4" t="n"/>
@@ -562,7 +562,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>TO%%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
+          <t>TO%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
@@ -582,7 +582,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>ORB%%: offensive rebounds / (own ORB + opponent DRB)</t>
+          <t>ORB%: offensive rebounds / (own ORB + opponent DRB)</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>eFG%%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
+          <t>eFG%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
         </is>
       </c>
       <c r="E11" s="4" t="n"/>
@@ -712,7 +712,7 @@
     <row r="13">
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>TO%%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
+          <t>TO%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
         </is>
       </c>
       <c r="E13" s="4" t="n"/>
@@ -721,7 +721,7 @@
     <row r="14">
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>ORB%%: offensive rebounds / (own ORB + opponent DRB)</t>
+          <t>ORB%: offensive rebounds / (own ORB + opponent DRB)</t>
         </is>
       </c>
       <c r="E14" s="4" t="n"/>

</xml_diff>

<commit_message>
Show one percent sign on the four-factors labels (#15)
The eFG, turnover and offensive rebound rows read with a doubled percent sign,
which looked like a typo in the sheet students are asked to trust.
</commit_message>
<xml_diff>
--- a/weeks/week04/data/hand-build-descriptive-worksheet.xlsx
+++ b/weeks/week04/data/hand-build-descriptive-worksheet.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>eFG%%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
+          <t>eFG%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
         </is>
       </c>
       <c r="E3" s="4" t="n"/>
@@ -562,7 +562,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>TO%%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
+          <t>TO%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
@@ -582,7 +582,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>ORB%%: offensive rebounds / (own ORB + opponent DRB)</t>
+          <t>ORB%: offensive rebounds / (own ORB + opponent DRB)</t>
         </is>
       </c>
       <c r="E6" s="4" t="n"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>eFG%%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
+          <t>eFG%: effective field goal percentage, (FG + 0.5 x 3P) / FGA</t>
         </is>
       </c>
       <c r="E11" s="4" t="n"/>
@@ -712,7 +712,7 @@
     <row r="13">
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>TO%%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
+          <t>TO%: turnovers per possession-ending event, TOV / (FGA + 0.44 x FTA + TOV)</t>
         </is>
       </c>
       <c r="E13" s="4" t="n"/>
@@ -721,7 +721,7 @@
     <row r="14">
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>ORB%%: offensive rebounds / (own ORB + opponent DRB)</t>
+          <t>ORB%: offensive rebounds / (own ORB + opponent DRB)</t>
         </is>
       </c>
       <c r="E14" s="4" t="n"/>

</xml_diff>